<commit_message>
now stores highelapsed time to xlsx files in HighElapsedTime folder and fixed order of date on dor sheet
</commit_message>
<xml_diff>
--- a/Individual Keyed Pass per User - Excel REPH - 2025-01-01.xlsx
+++ b/Individual Keyed Pass per User - Excel REPH - 2025-01-01.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python Projects\Ms drei app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14681E9E-F25A-48B2-B649-C774ADB0DEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820DD275-240F-4713-8312-F8D7C7B3C687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DC3DA337-D47D-435C-9FBD-49D8F17EF3E1}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="19">
   <si>
     <t>Formacion, Eric John</t>
   </si>
@@ -71,10 +71,37 @@
     <t>Username</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Work Type</t>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>REPORT ID</t>
+  </si>
+  <si>
+    <t>1=AUTO EXTRACTED</t>
+  </si>
+  <si>
+    <t>CREATION DATE</t>
+  </si>
+  <si>
+    <t>KEYING START DATE</t>
+  </si>
+  <si>
+    <t>KEYING END DATE</t>
+  </si>
+  <si>
+    <t>ELAPSED TIME</t>
+  </si>
+  <si>
+    <t>WORK TYPE</t>
+  </si>
+  <si>
+    <t>FORM &amp; PASS TYPE</t>
+  </si>
+  <si>
+    <t>STATE</t>
+  </si>
+  <si>
+    <t>AGENCY</t>
   </si>
 </sst>
 </file>
@@ -85,7 +112,7 @@
     <numFmt numFmtId="164" formatCode="0_);\(0\)"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy&quot;  &quot;h\:mm\:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,13 +120,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -114,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -127,6 +168,14 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -566,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3C8414-3AF4-458A-89B3-F4156E745445}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -574,7 +623,7 @@
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="2.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
@@ -585,11 +634,38 @@
       <c r="A1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
+      <c r="C1" s="5" t="s">
         <v>9</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -612,7 +688,7 @@
         <v>45658.205497685187</v>
       </c>
       <c r="H2" s="4">
-        <v>0.7</v>
+        <v>999</v>
       </c>
       <c r="I2" t="s">
         <v>1</v>
@@ -647,7 +723,7 @@
         <v>45658.20648148148</v>
       </c>
       <c r="H3" s="4">
-        <v>1.4</v>
+        <v>999</v>
       </c>
       <c r="I3" t="s">
         <v>1</v>
@@ -682,7 +758,7 @@
         <v>45658.210150462961</v>
       </c>
       <c r="H4" s="4">
-        <v>5.25</v>
+        <v>999</v>
       </c>
       <c r="I4" t="s">
         <v>1</v>
@@ -697,8 +773,218 @@
         <v>6</v>
       </c>
     </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1266850799</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
+        <v>45658.146064814813</v>
+      </c>
+      <c r="F5" s="3">
+        <v>45658.205011574071</v>
+      </c>
+      <c r="G5" s="3">
+        <v>45658.205497685187</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1266850809</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>45658.146134259259</v>
+      </c>
+      <c r="F6" s="3">
+        <v>45658.205509259256</v>
+      </c>
+      <c r="G6" s="3">
+        <v>45658.20648148148</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>2</v>
+      </c>
+      <c r="K6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1266855749</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>45658.163321759261</v>
+      </c>
+      <c r="F7" s="3">
+        <v>45658.206504629627</v>
+      </c>
+      <c r="G7" s="3">
+        <v>45658.210150462961</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1266850799</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3">
+        <v>45658.146064814813</v>
+      </c>
+      <c r="F8" s="3">
+        <v>45658.205011574071</v>
+      </c>
+      <c r="G8" s="3">
+        <v>45658.205497685187</v>
+      </c>
+      <c r="H8" s="4">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
+        <v>2</v>
+      </c>
+      <c r="K8" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1266850809</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3">
+        <v>45658.146134259259</v>
+      </c>
+      <c r="F9" s="3">
+        <v>45658.205509259256</v>
+      </c>
+      <c r="G9" s="3">
+        <v>45658.20648148148</v>
+      </c>
+      <c r="H9" s="4">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" t="s">
+        <v>3</v>
+      </c>
+      <c r="L9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1266855749</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>45658.163321759261</v>
+      </c>
+      <c r="F10" s="3">
+        <v>45658.206504629627</v>
+      </c>
+      <c r="G10" s="3">
+        <v>45658.210150462961</v>
+      </c>
+      <c r="H10" s="4">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>2</v>
+      </c>
+      <c r="K10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L10" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B4">
+  <conditionalFormatting sqref="B2:B10">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>SUMPRODUCT(--(TRIM($C2)=TRIM(SupervisorList)))&gt;0</formula>
     </cfRule>

</xml_diff>